<commit_message>
Comments + Upvotes Added. Security Updates Made Changes to 2FA
</commit_message>
<xml_diff>
--- a/Day_Scholars_Requests.xlsx
+++ b/Day_Scholars_Requests.xlsx
@@ -573,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -616,10 +616,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="str">
-        <v>OpenRoom</v>
+        <v>Random_3</v>
       </c>
       <c r="C2" s="6" t="str">
-        <v>student.openroom@gmail.com</v>
+        <v>random3@example.com</v>
       </c>
       <c r="D2" s="6" t="str">
         <v>N/A</v>
@@ -628,13 +628,13 @@
         <v>APPROVED</v>
       </c>
       <c r="F2" s="6" t="str">
-        <v>openroom@openroom.xyz</v>
+        <v>random3@openroom.xyz</v>
       </c>
       <c r="G2" s="6" t="str">
-        <v>123456</v>
+        <v>random3</v>
       </c>
       <c r="H2" s="6" t="str">
-        <v>21/8/2026, 6:40:51 pm</v>
+        <v>21/8/2026, 8:03:07 pm</v>
       </c>
     </row>
     <row r="3">
@@ -642,25 +642,25 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="str">
-        <v>Parth</v>
+        <v>Random_2</v>
       </c>
       <c r="C3" s="6" t="str">
-        <v>parth123.@example.com</v>
+        <v>random2@example.com</v>
       </c>
       <c r="D3" s="6" t="str">
         <v>N/A</v>
       </c>
-      <c r="E3" s="8" t="str">
-        <v>PENDING</v>
+      <c r="E3" s="7" t="str">
+        <v>APPROVED</v>
       </c>
       <c r="F3" s="6" t="str">
-        <v>—</v>
+        <v>random2@openroom.xyz</v>
       </c>
       <c r="G3" s="6" t="str">
-        <v>—</v>
+        <v>random2</v>
       </c>
       <c r="H3" s="6" t="str">
-        <v>21/8/2026, 6:37:29 pm</v>
+        <v>21/8/2026, 8:02:50 pm</v>
       </c>
     </row>
     <row r="4">
@@ -668,30 +668,108 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="str">
-        <v>Parth Bishnoi</v>
+        <v>Random_1</v>
       </c>
       <c r="C4" s="6" t="str">
-        <v>parthbishnoi05082000@gmail.com</v>
+        <v>random1@example.com</v>
       </c>
       <c r="D4" s="6" t="str">
         <v>N/A</v>
       </c>
-      <c r="E4" s="8" t="str">
+      <c r="E4" s="7" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="F4" s="6" t="str">
+        <v>random1@openroom.xyz</v>
+      </c>
+      <c r="G4" s="6" t="str">
+        <v>random2</v>
+      </c>
+      <c r="H4" s="6" t="str">
+        <v>21/8/2026, 8:02:40 pm</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="str">
+        <v>OpenRoom</v>
+      </c>
+      <c r="C5" s="6" t="str">
+        <v>student.openroom@gmail.com</v>
+      </c>
+      <c r="D5" s="6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E5" s="7" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="F5" s="6" t="str">
+        <v>openroom@openroom.xyz</v>
+      </c>
+      <c r="G5" s="6" t="str">
+        <v>123456</v>
+      </c>
+      <c r="H5" s="6" t="str">
+        <v>21/8/2026, 6:40:51 pm</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="str">
+        <v>Parth</v>
+      </c>
+      <c r="C6" s="6" t="str">
+        <v>parth123.@example.com</v>
+      </c>
+      <c r="D6" s="6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E6" s="8" t="str">
         <v>PENDING</v>
       </c>
-      <c r="F4" s="6" t="str">
+      <c r="F6" s="6" t="str">
         <v>—</v>
       </c>
-      <c r="G4" s="6" t="str">
+      <c r="G6" s="6" t="str">
         <v>—</v>
       </c>
-      <c r="H4" s="6" t="str">
+      <c r="H6" s="6" t="str">
+        <v>21/8/2026, 6:37:29 pm</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="str">
+        <v>Parth Bishnoi</v>
+      </c>
+      <c r="C7" s="6" t="str">
+        <v>parthbishnoi05082000@gmail.com</v>
+      </c>
+      <c r="D7" s="6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E7" s="8" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="F7" s="6" t="str">
+        <v>—</v>
+      </c>
+      <c r="G7" s="6" t="str">
+        <v>—</v>
+      </c>
+      <c r="H7" s="6" t="str">
         <v>21/8/2026, 5:10:30 pm</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Password Reset Feature for Users
</commit_message>
<xml_diff>
--- a/Day_Scholars_Requests.xlsx
+++ b/Day_Scholars_Requests.xlsx
@@ -573,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H11"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -616,10 +616,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="str">
-        <v>Random_3</v>
+        <v>Parth Bishnoi</v>
       </c>
       <c r="C2" s="6" t="str">
-        <v>random3@example.com</v>
+        <v>parthbishnoi0109@gmail.com</v>
       </c>
       <c r="D2" s="6" t="str">
         <v>N/A</v>
@@ -628,13 +628,13 @@
         <v>APPROVED</v>
       </c>
       <c r="F2" s="6" t="str">
-        <v>random3@openroom.xyz</v>
+        <v>parthbishnoi@openroom.xyz</v>
       </c>
       <c r="G2" s="6" t="str">
-        <v>random3</v>
+        <v>Parth123</v>
       </c>
       <c r="H2" s="6" t="str">
-        <v>21/8/2026, 8:03:07 pm</v>
+        <v>22/8/2026, 2:47:46 pm</v>
       </c>
     </row>
     <row r="3">
@@ -642,10 +642,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="str">
-        <v>Random_2</v>
+        <v>Parth Bishnoi</v>
       </c>
       <c r="C3" s="6" t="str">
-        <v>random2@example.com</v>
+        <v>parth.bishnoi@criskoco.in</v>
       </c>
       <c r="D3" s="6" t="str">
         <v>N/A</v>
@@ -654,13 +654,13 @@
         <v>APPROVED</v>
       </c>
       <c r="F3" s="6" t="str">
-        <v>random2@openroom.xyz</v>
+        <v>parth.bishnoi@openroom.xyz</v>
       </c>
       <c r="G3" s="6" t="str">
-        <v>random2</v>
+        <v>Parth@1234</v>
       </c>
       <c r="H3" s="6" t="str">
-        <v>21/8/2026, 8:02:50 pm</v>
+        <v>22/8/2026, 2:39:28 pm</v>
       </c>
     </row>
     <row r="4">
@@ -668,10 +668,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="str">
-        <v>Random_1</v>
+        <v>Maanya Goswami</v>
       </c>
       <c r="C4" s="6" t="str">
-        <v>random1@example.com</v>
+        <v>manya.goswami@openroom.xyz</v>
       </c>
       <c r="D4" s="6" t="str">
         <v>N/A</v>
@@ -680,13 +680,13 @@
         <v>APPROVED</v>
       </c>
       <c r="F4" s="6" t="str">
-        <v>random1@openroom.xyz</v>
+        <v>maanya.goswami@openroom.edu</v>
       </c>
       <c r="G4" s="6" t="str">
-        <v>random2</v>
+        <v>Maanya@1234</v>
       </c>
       <c r="H4" s="6" t="str">
-        <v>21/8/2026, 8:02:40 pm</v>
+        <v>22/8/2026, 2:25:57 pm</v>
       </c>
     </row>
     <row r="5">
@@ -694,25 +694,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="str">
-        <v>OpenRoom</v>
+        <v>Maanya Goswami</v>
       </c>
       <c r="C5" s="6" t="str">
-        <v>student.openroom@gmail.com</v>
+        <v>manya.goswami@openroom.xyz</v>
       </c>
       <c r="D5" s="6" t="str">
         <v>N/A</v>
       </c>
-      <c r="E5" s="7" t="str">
-        <v>APPROVED</v>
+      <c r="E5" s="8" t="str">
+        <v>PENDING</v>
       </c>
       <c r="F5" s="6" t="str">
-        <v>openroom@openroom.xyz</v>
+        <v>—</v>
       </c>
       <c r="G5" s="6" t="str">
-        <v>123456</v>
+        <v>—</v>
       </c>
       <c r="H5" s="6" t="str">
-        <v>21/8/2026, 6:40:51 pm</v>
+        <v>22/8/2026, 2:25:55 pm</v>
       </c>
     </row>
     <row r="6">
@@ -720,25 +720,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="str">
-        <v>Parth</v>
+        <v>Random_3</v>
       </c>
       <c r="C6" s="6" t="str">
-        <v>parth123.@example.com</v>
+        <v>random3@example.com</v>
       </c>
       <c r="D6" s="6" t="str">
         <v>N/A</v>
       </c>
-      <c r="E6" s="8" t="str">
-        <v>PENDING</v>
+      <c r="E6" s="7" t="str">
+        <v>APPROVED</v>
       </c>
       <c r="F6" s="6" t="str">
-        <v>—</v>
+        <v>random3@openroom.xyz</v>
       </c>
       <c r="G6" s="6" t="str">
-        <v>—</v>
+        <v>random3</v>
       </c>
       <c r="H6" s="6" t="str">
-        <v>21/8/2026, 6:37:29 pm</v>
+        <v>21/8/2026, 8:03:07 pm</v>
       </c>
     </row>
     <row r="7">
@@ -746,30 +746,134 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="str">
+        <v>Random_2</v>
+      </c>
+      <c r="C7" s="6" t="str">
+        <v>random2@example.com</v>
+      </c>
+      <c r="D7" s="6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E7" s="7" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="F7" s="6" t="str">
+        <v>random2@openroom.xyz</v>
+      </c>
+      <c r="G7" s="6" t="str">
+        <v>random2</v>
+      </c>
+      <c r="H7" s="6" t="str">
+        <v>21/8/2026, 8:02:50 pm</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="str">
+        <v>Random_1</v>
+      </c>
+      <c r="C8" s="6" t="str">
+        <v>random1@example.com</v>
+      </c>
+      <c r="D8" s="6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E8" s="7" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="F8" s="6" t="str">
+        <v>random1@openroom.xyz</v>
+      </c>
+      <c r="G8" s="6" t="str">
+        <v>random2</v>
+      </c>
+      <c r="H8" s="6" t="str">
+        <v>21/8/2026, 8:02:40 pm</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="str">
+        <v>OpenRoom</v>
+      </c>
+      <c r="C9" s="6" t="str">
+        <v>student.openroom@gmail.com</v>
+      </c>
+      <c r="D9" s="6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E9" s="7" t="str">
+        <v>APPROVED</v>
+      </c>
+      <c r="F9" s="6" t="str">
+        <v>openroom@openroom.xyz</v>
+      </c>
+      <c r="G9" s="6" t="str">
+        <v>123456</v>
+      </c>
+      <c r="H9" s="6" t="str">
+        <v>21/8/2026, 6:40:51 pm</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="str">
+        <v>Parth</v>
+      </c>
+      <c r="C10" s="6" t="str">
+        <v>parth123.@example.com</v>
+      </c>
+      <c r="D10" s="6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E10" s="8" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="F10" s="6" t="str">
+        <v>—</v>
+      </c>
+      <c r="G10" s="6" t="str">
+        <v>—</v>
+      </c>
+      <c r="H10" s="6" t="str">
+        <v>21/8/2026, 6:37:29 pm</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="str">
         <v>Parth Bishnoi</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C11" s="6" t="str">
         <v>parthbishnoi05082000@gmail.com</v>
       </c>
-      <c r="D7" s="6" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="E7" s="8" t="str">
+      <c r="D11" s="6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E11" s="8" t="str">
         <v>PENDING</v>
       </c>
-      <c r="F7" s="6" t="str">
+      <c r="F11" s="6" t="str">
         <v>—</v>
       </c>
-      <c r="G7" s="6" t="str">
+      <c r="G11" s="6" t="str">
         <v>—</v>
       </c>
-      <c r="H7" s="6" t="str">
+      <c r="H11" s="6" t="str">
         <v>21/8/2026, 5:10:30 pm</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>